<commit_message>
docs(hw03): verify external evidence and finalize reports
</commit_message>
<xml_diff>
--- a/docs/assignments/HW03/deliverables/usability/usability_results.xlsx
+++ b/docs/assignments/HW03/deliverables/usability/usability_results.xlsx
@@ -649,7 +649,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -835,7 +835,7 @@
       </c>
       <c r="J3" s="11">
         <f>SUS!M2</f>
-        <v>75</v>
+        <v/>
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
       </c>
       <c r="J4" s="8">
         <f>SUS!M3</f>
-        <v>82.5</v>
+        <v/>
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
       </c>
       <c r="J5" s="11">
         <f>SUS!M4</f>
-        <v>67.5</v>
+        <v/>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="J6" s="8">
         <f>SUS!M5</f>
-        <v>67.5</v>
+        <v/>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="J7" s="11">
         <f>SUS!M6</f>
-        <v>77.5</v>
+        <v/>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="J8" s="8">
         <f>SUS!M7</f>
-        <v>75</v>
+        <v/>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="J9" s="11">
         <f>SUS!M8</f>
-        <v>70</v>
+        <v/>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3936,7 +3936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4095,11 +4095,11 @@
       </c>
       <c r="L2" s="8">
         <f>IF(COUNTA(B2:K2)=0,"",IF(COUNTA(B2:K2)&lt;10,"INCOMPLETE",SUM(B2-1,5-C2,D2-1,5-E2,F2-1,5-G2,H2-1,5-I2,J2-1,5-K2)))</f>
-        <v>30</v>
+        <v/>
       </c>
       <c r="M2" s="9">
         <f>IF(ISNUMBER(L2),L2*2.5,"")</f>
-        <v>75</v>
+        <v/>
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="L3" s="11">
         <f>IF(COUNTA(B3:K3)=0,"",IF(COUNTA(B3:K3)&lt;10,"INCOMPLETE",SUM(B3-1,5-C3,D3-1,5-E3,F3-1,5-G3,H3-1,5-I3,J3-1,5-K3)))</f>
-        <v>33</v>
+        <v/>
       </c>
       <c r="M3" s="12">
         <f>IF(ISNUMBER(L3),L3*2.5,"")</f>
-        <v>82.5</v>
+        <v/>
       </c>
       <c r="N3" s="11" t="inlineStr">
         <is>
@@ -4233,11 +4233,11 @@
       </c>
       <c r="L4" s="8">
         <f>IF(COUNTA(B4:K4)=0,"",IF(COUNTA(B4:K4)&lt;10,"INCOMPLETE",SUM(B4-1,5-C4,D4-1,5-E4,F4-1,5-G4,H4-1,5-I4,J4-1,5-K4)))</f>
-        <v>27</v>
+        <v/>
       </c>
       <c r="M4" s="9">
         <f>IF(ISNUMBER(L4),L4*2.5,"")</f>
-        <v>67.5</v>
+        <v/>
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
@@ -4302,11 +4302,11 @@
       </c>
       <c r="L5" s="11">
         <f>IF(COUNTA(B5:K5)=0,"",IF(COUNTA(B5:K5)&lt;10,"INCOMPLETE",SUM(B5-1,5-C5,D5-1,5-E5,F5-1,5-G5,H5-1,5-I5,J5-1,5-K5)))</f>
-        <v>27</v>
+        <v/>
       </c>
       <c r="M5" s="12">
         <f>IF(ISNUMBER(L5),L5*2.5,"")</f>
-        <v>67.5</v>
+        <v/>
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
@@ -4371,11 +4371,11 @@
       </c>
       <c r="L6" s="8">
         <f>IF(COUNTA(B6:K6)=0,"",IF(COUNTA(B6:K6)&lt;10,"INCOMPLETE",SUM(B6-1,5-C6,D6-1,5-E6,F6-1,5-G6,H6-1,5-I6,J6-1,5-K6)))</f>
-        <v>31</v>
+        <v/>
       </c>
       <c r="M6" s="9">
         <f>IF(ISNUMBER(L6),L6*2.5,"")</f>
-        <v>77.5</v>
+        <v/>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
@@ -4440,11 +4440,11 @@
       </c>
       <c r="L7" s="11">
         <f>IF(COUNTA(B7:K7)=0,"",IF(COUNTA(B7:K7)&lt;10,"INCOMPLETE",SUM(B7-1,5-C7,D7-1,5-E7,F7-1,5-G7,H7-1,5-I7,J7-1,5-K7)))</f>
-        <v>30</v>
+        <v/>
       </c>
       <c r="M7" s="12">
         <f>IF(ISNUMBER(L7),L7*2.5,"")</f>
-        <v>75</v>
+        <v/>
       </c>
       <c r="N7" s="11" t="inlineStr">
         <is>
@@ -4509,11 +4509,11 @@
       </c>
       <c r="L8" s="8">
         <f>IF(COUNTA(B8:K8)=0,"",IF(COUNTA(B8:K8)&lt;10,"INCOMPLETE",SUM(B8-1,5-C8,D8-1,5-E8,F8-1,5-G8,H8-1,5-I8,J8-1,5-K8)))</f>
-        <v>28</v>
+        <v/>
       </c>
       <c r="M8" s="9">
         <f>IF(ISNUMBER(L8),L8*2.5,"")</f>
-        <v>70</v>
+        <v/>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
@@ -4559,7 +4559,7 @@
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="12">
         <f>AVERAGE(M2:M8)</f>
-        <v>73.57142857142857</v>
+        <v/>
       </c>
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
@@ -4595,7 +4595,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4713,12 +4713,12 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -4761,12 +4761,12 @@
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -4809,12 +4809,12 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -4857,12 +4857,12 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -4905,12 +4905,12 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -4953,12 +4953,12 @@
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -5001,12 +5001,12 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>
@@ -5049,12 +5049,12 @@
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>Not independently verified</t>
+          <t>Yes - publicly listed</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>Local file verified; shared Drive folder supplied</t>
+          <t>Local file and public Drive listing verified on 3 August 2026</t>
         </is>
       </c>
     </row>

</xml_diff>